<commit_message>
Stage 3: density group difference rerun on revised data
</commit_message>
<xml_diff>
--- a/results/density_group_difference/density_sensitivity_results.xlsx
+++ b/results/density_group_difference/density_sensitivity_results.xlsx
@@ -58,19 +58,19 @@
     <t xml:space="preserve">+ Age at MRI</t>
   </si>
   <si>
-    <t xml:space="preserve">0.0056</t>
+    <t xml:space="preserve">0.0027</t>
   </si>
   <si>
     <t xml:space="preserve">+ Sex</t>
   </si>
   <si>
-    <t xml:space="preserve">0.0015</t>
+    <t xml:space="preserve">0.0011</t>
   </si>
   <si>
     <t xml:space="preserve">+ Relative motion</t>
   </si>
   <si>
-    <t xml:space="preserve">0.0206</t>
+    <t xml:space="preserve">0.0025</t>
   </si>
   <si>
     <t xml:space="preserve">+ eTIV</t>
@@ -82,16 +82,16 @@
     <t xml:space="preserve">Excl. outliers (2 SD)</t>
   </si>
   <si>
-    <t xml:space="preserve">0.0030</t>
-  </si>
-  <si>
-    <t xml:space="preserve">0.0100</t>
-  </si>
-  <si>
-    <t xml:space="preserve">0.0027</t>
-  </si>
-  <si>
-    <t xml:space="preserve">0.0470</t>
+    <t xml:space="preserve">0.0028</t>
+  </si>
+  <si>
+    <t xml:space="preserve">0.0078</t>
+  </si>
+  <si>
+    <t xml:space="preserve">0.0020</t>
+  </si>
+  <si>
+    <t xml:space="preserve">0.0073</t>
   </si>
   <si>
     <t xml:space="preserve">Variable</t>
@@ -569,14 +569,14 @@
       </c>
       <c r="E2" s="2"/>
       <c r="F2" s="2" t="n">
-        <v>3.79</v>
+        <v>3.86</v>
       </c>
       <c r="G2" s="2" t="s">
         <v>12</v>
       </c>
       <c r="H2" s="2"/>
       <c r="I2" s="2" t="n">
-        <v>-0.48</v>
+        <v>-0.492</v>
       </c>
       <c r="J2" s="2"/>
     </row>
@@ -594,20 +594,20 @@
         <v>45</v>
       </c>
       <c r="E3" s="2" t="n">
-        <v>-0.0132</v>
+        <v>-0.0133</v>
       </c>
       <c r="F3" s="2" t="n">
-        <v>-2.8</v>
+        <v>-3.04</v>
       </c>
       <c r="G3" s="2" t="s">
         <v>14</v>
       </c>
       <c r="H3" s="2" t="n">
-        <v>0.035</v>
+        <v>0.041</v>
       </c>
       <c r="I3" s="2"/>
       <c r="J3" s="2" t="n">
-        <v>0.037</v>
+        <v>0.043</v>
       </c>
     </row>
     <row r="4">
@@ -624,20 +624,20 @@
         <v>45</v>
       </c>
       <c r="E4" s="2" t="n">
-        <v>-0.0146</v>
+        <v>-0.0139</v>
       </c>
       <c r="F4" s="2" t="n">
-        <v>-3.22</v>
+        <v>-3.31</v>
       </c>
       <c r="G4" s="2" t="s">
         <v>16</v>
       </c>
       <c r="H4" s="2" t="n">
-        <v>0.046</v>
+        <v>0.049</v>
       </c>
       <c r="I4" s="2"/>
       <c r="J4" s="2" t="n">
-        <v>0.105</v>
+        <v>0.11</v>
       </c>
     </row>
     <row r="5">
@@ -654,16 +654,16 @@
         <v>45</v>
       </c>
       <c r="E5" s="2" t="n">
-        <v>-0.0116</v>
+        <v>-0.014</v>
       </c>
       <c r="F5" s="2" t="n">
-        <v>-2.33</v>
+        <v>-3.06</v>
       </c>
       <c r="G5" s="2" t="s">
         <v>18</v>
       </c>
       <c r="H5" s="2" t="n">
-        <v>0.025</v>
+        <v>0.042</v>
       </c>
       <c r="I5" s="2"/>
       <c r="J5" s="2" t="n">
@@ -684,20 +684,20 @@
         <v>45</v>
       </c>
       <c r="E6" s="2" t="n">
-        <v>-0.0152</v>
+        <v>-0.0146</v>
       </c>
       <c r="F6" s="2" t="n">
-        <v>-3.46</v>
+        <v>-3.59</v>
       </c>
       <c r="G6" s="2" t="s">
         <v>12</v>
       </c>
       <c r="H6" s="2" t="n">
-        <v>0.053</v>
+        <v>0.057</v>
       </c>
       <c r="I6" s="2"/>
       <c r="J6" s="2" t="n">
-        <v>0.151</v>
+        <v>0.167</v>
       </c>
     </row>
     <row r="7">
@@ -714,20 +714,20 @@
         <v>45</v>
       </c>
       <c r="E7" s="2" t="n">
-        <v>-0.0161</v>
+        <v>-0.0163</v>
       </c>
       <c r="F7" s="2" t="n">
-        <v>-3.37</v>
+        <v>-3.82</v>
       </c>
       <c r="G7" s="2" t="s">
         <v>12</v>
       </c>
       <c r="H7" s="2" t="n">
-        <v>0.051</v>
+        <v>0.065</v>
       </c>
       <c r="I7" s="2"/>
       <c r="J7" s="2" t="n">
-        <v>0.164</v>
+        <v>0.186</v>
       </c>
     </row>
     <row r="8">
@@ -738,21 +738,21 @@
         <v>11</v>
       </c>
       <c r="C8" s="2" t="n">
-        <v>165</v>
+        <v>164</v>
       </c>
       <c r="D8" s="2" t="n">
         <v>45</v>
       </c>
       <c r="E8" s="2"/>
       <c r="F8" s="2" t="n">
-        <v>3.06</v>
+        <v>3.07</v>
       </c>
       <c r="G8" s="2" t="s">
         <v>22</v>
       </c>
       <c r="H8" s="2"/>
       <c r="I8" s="2" t="n">
-        <v>-0.449</v>
+        <v>-0.455</v>
       </c>
       <c r="J8" s="2"/>
     </row>
@@ -764,22 +764,22 @@
         <v>13</v>
       </c>
       <c r="C9" s="2" t="n">
-        <v>165</v>
+        <v>164</v>
       </c>
       <c r="D9" s="2" t="n">
         <v>45</v>
       </c>
       <c r="E9" s="2" t="n">
-        <v>-0.0097</v>
+        <v>-0.0094</v>
       </c>
       <c r="F9" s="2" t="n">
-        <v>-2.6</v>
+        <v>-2.69</v>
       </c>
       <c r="G9" s="2" t="s">
         <v>23</v>
       </c>
       <c r="H9" s="2" t="n">
-        <v>0.032</v>
+        <v>0.034</v>
       </c>
       <c r="I9" s="2"/>
       <c r="J9" s="2" t="n">
@@ -794,26 +794,26 @@
         <v>15</v>
       </c>
       <c r="C10" s="2" t="n">
-        <v>165</v>
+        <v>164</v>
       </c>
       <c r="D10" s="2" t="n">
         <v>45</v>
       </c>
       <c r="E10" s="2" t="n">
-        <v>-0.0109</v>
+        <v>-0.0104</v>
       </c>
       <c r="F10" s="2" t="n">
-        <v>-3.04</v>
+        <v>-3.13</v>
       </c>
       <c r="G10" s="2" t="s">
         <v>24</v>
       </c>
       <c r="H10" s="2" t="n">
-        <v>0.043</v>
+        <v>0.045</v>
       </c>
       <c r="I10" s="2"/>
       <c r="J10" s="2" t="n">
-        <v>0.099</v>
+        <v>0.116</v>
       </c>
     </row>
     <row r="11">
@@ -824,26 +824,26 @@
         <v>17</v>
       </c>
       <c r="C11" s="2" t="n">
-        <v>165</v>
+        <v>164</v>
       </c>
       <c r="D11" s="2" t="n">
         <v>45</v>
       </c>
       <c r="E11" s="2" t="n">
-        <v>-0.0079</v>
+        <v>-0.0099</v>
       </c>
       <c r="F11" s="2" t="n">
-        <v>-2</v>
+        <v>-2.71</v>
       </c>
       <c r="G11" s="2" t="s">
         <v>25</v>
       </c>
       <c r="H11" s="2" t="n">
-        <v>0.019</v>
+        <v>0.034</v>
       </c>
       <c r="I11" s="2"/>
       <c r="J11" s="2" t="n">
-        <v>0.043</v>
+        <v>0.035</v>
       </c>
     </row>
     <row r="12">
@@ -854,26 +854,26 @@
         <v>19</v>
       </c>
       <c r="C12" s="2" t="n">
-        <v>165</v>
+        <v>164</v>
       </c>
       <c r="D12" s="2" t="n">
         <v>45</v>
       </c>
       <c r="E12" s="2" t="n">
-        <v>-0.0119</v>
+        <v>-0.0114</v>
       </c>
       <c r="F12" s="2" t="n">
-        <v>-3.6</v>
+        <v>-3.65</v>
       </c>
       <c r="G12" s="2" t="s">
         <v>12</v>
       </c>
       <c r="H12" s="2" t="n">
-        <v>0.059</v>
+        <v>0.061</v>
       </c>
       <c r="I12" s="2"/>
       <c r="J12" s="2" t="n">
-        <v>0.237</v>
+        <v>0.226</v>
       </c>
     </row>
     <row r="13">
@@ -884,26 +884,26 @@
         <v>20</v>
       </c>
       <c r="C13" s="2" t="n">
-        <v>165</v>
+        <v>164</v>
       </c>
       <c r="D13" s="2" t="n">
         <v>45</v>
       </c>
       <c r="E13" s="2" t="n">
-        <v>-0.0125</v>
+        <v>-0.0122</v>
       </c>
       <c r="F13" s="2" t="n">
-        <v>-3.46</v>
+        <v>-3.7</v>
       </c>
       <c r="G13" s="2" t="s">
         <v>12</v>
       </c>
       <c r="H13" s="2" t="n">
-        <v>0.055</v>
+        <v>0.063</v>
       </c>
       <c r="I13" s="2"/>
       <c r="J13" s="2" t="n">
-        <v>0.24</v>
+        <v>0.233</v>
       </c>
     </row>
   </sheetData>
@@ -953,16 +953,16 @@
         <v>171</v>
       </c>
       <c r="C2" t="n">
-        <v>0.9142</v>
+        <v>0.9152</v>
       </c>
       <c r="D2" t="n">
-        <v>0.0299</v>
+        <v>0.0278</v>
       </c>
       <c r="E2" t="n">
-        <v>0.7438</v>
+        <v>0.7441</v>
       </c>
       <c r="F2" t="n">
-        <v>0.9696</v>
+        <v>0.9748</v>
       </c>
     </row>
     <row r="3">
@@ -973,16 +973,16 @@
         <v>45</v>
       </c>
       <c r="C3" t="n">
-        <v>0.9276</v>
+        <v>0.928</v>
       </c>
       <c r="D3" t="n">
-        <v>0.0181</v>
+        <v>0.0171</v>
       </c>
       <c r="E3" t="n">
-        <v>0.8916</v>
+        <v>0.8939</v>
       </c>
       <c r="F3" t="n">
-        <v>0.9641</v>
+        <v>0.9613</v>
       </c>
     </row>
     <row r="4">
@@ -1033,16 +1033,16 @@
         <v>171</v>
       </c>
       <c r="C6" t="n">
-        <v>1.1206</v>
+        <v>0.5081</v>
       </c>
       <c r="D6" t="n">
-        <v>0.124</v>
+        <v>0.1607</v>
       </c>
       <c r="E6" t="n">
-        <v>0.7713</v>
+        <v>0.2152</v>
       </c>
       <c r="F6" t="n">
-        <v>1.4741</v>
+        <v>1.354</v>
       </c>
     </row>
     <row r="7">
@@ -1053,16 +1053,16 @@
         <v>45</v>
       </c>
       <c r="C7" t="n">
-        <v>1.0158</v>
+        <v>0.3912</v>
       </c>
       <c r="D7" t="n">
-        <v>0.0813</v>
+        <v>0.0975</v>
       </c>
       <c r="E7" t="n">
-        <v>0.8681</v>
+        <v>0.228</v>
       </c>
       <c r="F7" t="n">
-        <v>1.2242</v>
+        <v>0.7574</v>
       </c>
     </row>
     <row r="8">
@@ -1073,10 +1073,10 @@
         <v>171</v>
       </c>
       <c r="C8" t="n">
-        <v>1317474.1856</v>
+        <v>1316535.5823</v>
       </c>
       <c r="D8" t="n">
-        <v>153573.5208</v>
+        <v>153898.331</v>
       </c>
       <c r="E8" t="n">
         <v>952334.5791</v>
@@ -1093,10 +1093,10 @@
         <v>45</v>
       </c>
       <c r="C9" t="n">
-        <v>1346437.6529</v>
+        <v>1346021.8767</v>
       </c>
       <c r="D9" t="n">
-        <v>138495.709</v>
+        <v>138349.4287</v>
       </c>
       <c r="E9" t="n">
         <v>1080430.2507</v>
@@ -1152,10 +1152,10 @@
         <v>46</v>
       </c>
       <c r="C2" t="n">
-        <v>0.834480780263913</v>
+        <v>0.838496844520941</v>
       </c>
       <c r="D2" t="n">
-        <v>1.15756029591837</v>
+        <v>0.417987933580099</v>
       </c>
       <c r="E2" t="n">
         <v>1468155.468455</v>
@@ -1166,82 +1166,82 @@
     </row>
     <row r="3">
       <c r="A3" t="n">
-        <v>191</v>
+        <v>210</v>
       </c>
       <c r="B3" t="s">
         <v>46</v>
       </c>
       <c r="C3" t="n">
-        <v>0.804360298336202</v>
+        <v>0.848537005163511</v>
       </c>
       <c r="D3" t="n">
-        <v>1.42315710810811</v>
+        <v>0.52152456119703</v>
       </c>
       <c r="E3" t="n">
-        <v>1288092.6569</v>
+        <v>1564494.350423</v>
       </c>
       <c r="F3" t="n">
-        <v>5.7900185585022</v>
+        <v>5.59539604187012</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="n">
-        <v>210</v>
+        <v>337</v>
       </c>
       <c r="B4" t="s">
         <v>46</v>
       </c>
       <c r="C4" t="n">
-        <v>0.843086632243259</v>
+        <v>0.855995410212278</v>
       </c>
       <c r="D4" t="n">
-        <v>1.14834930864197</v>
+        <v>0.501040464224257</v>
       </c>
       <c r="E4" t="n">
-        <v>1564494.350423</v>
+        <v>1292269.879425</v>
       </c>
       <c r="F4" t="n">
-        <v>5.59539604187012</v>
+        <v>5.56790494918823</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="n">
-        <v>321</v>
+        <v>570</v>
       </c>
       <c r="B5" t="s">
         <v>46</v>
       </c>
       <c r="C5" t="n">
-        <v>0.826448651749857</v>
+        <v>0.839931153184165</v>
       </c>
       <c r="D5" t="n">
-        <v>1.04793379569892</v>
+        <v>0.61932439719802</v>
       </c>
       <c r="E5" t="n">
-        <v>1347522.975233</v>
+        <v>1461039.223315</v>
       </c>
       <c r="F5" t="n">
-        <v>5.71598386764526</v>
+        <v>5.44731664657593</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="n">
-        <v>337</v>
+        <v>645</v>
       </c>
       <c r="B6" t="s">
         <v>46</v>
       </c>
       <c r="C6" t="n">
-        <v>0.853413654618474</v>
+        <v>0.859150889271371</v>
       </c>
       <c r="D6" t="n">
-        <v>1.12331431914894</v>
+        <v>0.281407205580693</v>
       </c>
       <c r="E6" t="n">
-        <v>1292269.879425</v>
+        <v>1572050.832763</v>
       </c>
       <c r="F6" t="n">
-        <v>5.56790494918823</v>
+        <v>5.54326438903809</v>
       </c>
     </row>
     <row r="7">
@@ -1252,16 +1252,36 @@
         <v>46</v>
       </c>
       <c r="C7" t="n">
-        <v>0.743832472748135</v>
+        <v>0.74411933448078</v>
       </c>
       <c r="D7" t="n">
-        <v>0.908970282828283</v>
+        <v>0.377994620712079</v>
       </c>
       <c r="E7" t="n">
         <v>1112354.390655</v>
       </c>
       <c r="F7" t="n">
         <v>5.55711317062378</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="n">
+        <v>901</v>
+      </c>
+      <c r="B8" t="s">
+        <v>46</v>
+      </c>
+      <c r="C8" t="n">
+        <v>0.855995410212278</v>
+      </c>
+      <c r="D8" t="n">
+        <v>0.572082563210891</v>
+      </c>
+      <c r="E8" t="n">
+        <v>1376048.437381</v>
+      </c>
+      <c r="F8" t="n">
+        <v>5.52672433853149</v>
       </c>
     </row>
   </sheetData>

</xml_diff>